<commit_message>
✨ Add Xiao Sun's QR/banner and footer disclaimer
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/宣群资料/信息.xlsx
+++ b/宣群资料/信息.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\我的文件\ACA stuff\Wechat\宣群\宣群资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DC0C05C-D153-4978-A6AA-3AAA6BC15E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9EDD9C-5DD7-40FA-937C-0473C7416EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Form responses 1" sheetId="1" r:id="rId1"/>
@@ -2087,7 +2087,7 @@
     <col min="10" max="10" width="42" customWidth="1"/>
     <col min="11" max="11" width="36" customWidth="1"/>
     <col min="12" max="12" width="18.85546875" customWidth="1"/>
-    <col min="13" max="13" width="21.28515625" customWidth="1"/>
+    <col min="13" max="13" width="45.42578125" customWidth="1"/>
     <col min="14" max="20" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
✨ Update QR codes, add new group, fix mobile modal scroll
- Update QR images (Aoi_, im@s, 王浩711, 音游群) with cache-busting
- kotomi: switch from two QRs to a single QR
- Add ken's Arknights group (placeholder card)
- Fix modal overflow/scrolling on mobile for double-QR view

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/宣群资料/信息.xlsx
+++ b/宣群资料/信息.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\我的文件\ACA stuff\Wechat\宣群\宣群资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9EDD9C-5DD7-40FA-937C-0473C7416EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F5CBA4-E5C2-4700-B775-E3653B7F95AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Form responses 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="86">
   <si>
     <t>Email address</t>
   </si>
@@ -1632,13 +1632,25 @@
   <si>
     <t>港大跑团</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ken</t>
+  </si>
+  <si>
+    <t>二游交流, COS / 摄影 / 同人创作, 综合闲聊 / 吹水联络</t>
+  </si>
+  <si>
+    <t>鹰角网络相关游戏二创.日常抽象内容.番剧.galgame.日常大学生活聚餐等活动</t>
+  </si>
+  <si>
+    <t>重铸未来，方舟启航</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1741,6 +1753,13 @@
       <family val="2"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1771,7 +1790,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1789,6 +1808,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1857,7 +1877,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="C1:N10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="C1:N11">
   <tableColumns count="12">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email address"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="申请人微信昵称"/>
@@ -2077,7 +2097,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="4" width="18.85546875" customWidth="1"/>
@@ -2430,6 +2450,23 @@
         <v>70</v>
       </c>
     </row>
+    <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
✨ Add Ken's group name and QR code
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/宣群资料/信息.xlsx
+++ b/宣群资料/信息.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\我的文件\ACA stuff\Wechat\宣群\宣群资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F5CBA4-E5C2-4700-B775-E3653B7F95AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A38F198-DFDA-4D3B-A3D0-8392E850237D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="390" yWindow="390" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="87">
   <si>
     <t>Email address</t>
   </si>
@@ -1644,13 +1644,16 @@
   </si>
   <si>
     <t>重铸未来，方舟启航</t>
+  </si>
+  <si>
+    <t>龙门大学巴别塔分部</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1760,6 +1763,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1790,7 +1801,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1809,6 +1820,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2451,6 +2463,12 @@
       </c>
     </row>
     <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>86</v>
+      </c>
       <c r="D11" s="9" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
✨ Add Stronghold Protocol group
</commit_message>
<xml_diff>
--- a/宣群资料/信息.xlsx
+++ b/宣群资料/信息.xlsx
@@ -1241,8 +1241,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="10" t="n"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>qr 头图</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>重振卫戍协议荣光</t>
+        </is>
+      </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
           <t>|ω・）</t>
@@ -1288,7 +1296,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>更衣人偶坠入偶像</t>
+          <t>更衣人偶坠入港大</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">

</xml_diff>

<commit_message>
✨ Add WUWA1001 1A group
</commit_message>
<xml_diff>
--- a/宣群资料/信息.xlsx
+++ b/宣群资料/信息.xlsx
@@ -312,7 +312,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:N15" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:N16" headerRowCount="1">
   <tableColumns count="12">
     <tableColumn id="2" name="Email address"/>
     <tableColumn id="5" name="申请人微信昵称"/>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.81640625" customWidth="1" min="3" max="4"/>
@@ -1337,6 +1337,58 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>qr 头图</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>WUWA1001 1A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>mairisqiao1007@gmail.com</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>乔</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>13927753213</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>微信群</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>二游交流</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>同意入驻，支持 ACA 活动宣传</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>二游鸣潮同好交流</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>潮批来潮批从四面八方来</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId1"/>

</xml_diff>